<commit_message>
chore(attendance): record Oct 12-15 shifts and format omar_elnemr_attendance_october_2026.xlsx with standardized table style
</commit_message>
<xml_diff>
--- a/attendance_september_2026_standardized.xlsx
+++ b/attendance_september_2026_standardized.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Detailed Timesheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Team Leaderboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Timesheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Leaderboard" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Detailed Timesheet'!$A$1:$I$68</definedName>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3582,51 +3582,6 @@
       <c r="I68" s="3" t="inlineStr">
         <is>
           <t>Morning departure processing (8h 40m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Omar Elnemr</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G69" t="n">
-        <v>0</v>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>Automatic: No reply recorded (Day Off)</t>
         </is>
       </c>
     </row>

</xml_diff>